<commit_message>
Update evaluation logic to handle missing scores and enforce GPU 5 usage
</commit_message>
<xml_diff>
--- a/results/drama_results.xlsx
+++ b/results/drama_results.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runs" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results'!$A$1:$C$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Runs'!$A$1:$P$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results'!$A$1:$E$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Runs'!$A$1:$P$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -458,12 +458,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -478,7 +480,13 @@
         </is>
       </c>
       <c r="C1" s="1" t="n">
+        <v>2010</v>
+      </c>
+      <c r="D1" s="1" t="n">
         <v>3710</v>
+      </c>
+      <c r="E1" s="1" t="n">
+        <v>6010</v>
       </c>
     </row>
     <row r="2">
@@ -493,6 +501,12 @@
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>101.40</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -506,6 +520,12 @@
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>105.20</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -519,6 +539,12 @@
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>336.00</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -532,6 +558,12 @@
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>630.00</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -545,6 +577,12 @@
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>14000.00</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -558,6 +596,12 @@
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>5800.00</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -570,11 +614,13 @@
           <t>X</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>1250.00</t>
         </is>
       </c>
+      <c r="E8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -587,16 +633,18 @@
           <t>O</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>1430.00</t>
         </is>
       </c>
+      <c r="E9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Frostbite</t>
+          <t>Jamesbond</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -605,11 +653,17 @@
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>355.00</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Frostbite</t>
+          <t>Jamesbond</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -618,11 +672,13 @@
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Jamesbond</t>
+          <t>Pong</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -632,14 +688,16 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>355.00</t>
-        </is>
-      </c>
+          <t>20.00</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Jamesbond</t>
+          <t>Pong</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -647,12 +705,18 @@
           <t>O</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>20.00</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Krull</t>
+          <t>Qbert</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -661,11 +725,17 @@
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>787.50</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Krull</t>
+          <t>Qbert</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -674,11 +744,17 @@
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>792.50</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Pong</t>
+          <t>UpNDown</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -687,11 +763,17 @@
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2654.00</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Pong</t>
+          <t>UpNDown</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -700,73 +782,11 @@
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Qbert</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>787.50</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Qbert</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>792.50</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>UpNDown</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>2654.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>UpNDown</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C21"/>
+  <autoFilter ref="A1:E17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -777,7 +797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -883,12 +903,12 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Mamba2_AC_Krull_seed6010_X</t>
+          <t>Mamba2_AC_Assault_seed6010_X</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>mera5ngk</t>
+          <t>ds19f3ml</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -908,7 +928,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Krull</t>
+          <t>Assault</t>
         </is>
       </c>
       <c r="G2" s="3" t="n">
@@ -919,7 +939,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr"/>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>336.00</t>
+        </is>
+      </c>
       <c r="J2" s="3" t="inlineStr"/>
       <c r="K2" s="3" t="n">
         <v>50000</v>
@@ -939,18 +963,18 @@
         <v>0.0625</v>
       </c>
       <c r="P2" s="4" t="n">
-        <v>46277.48331018518</v>
+        <v>46277.48542824074</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Mamba2_AC_Frostbite_seed6010_X</t>
+          <t>Mamba2_AC_Amidar_seed6010_X</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>kwxa3efq</t>
+          <t>d2x1c1en</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -970,7 +994,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Frostbite</t>
+          <t>Amidar</t>
         </is>
       </c>
       <c r="G3" s="3" t="n">
@@ -1001,18 +1025,18 @@
         <v>0.0625</v>
       </c>
       <c r="P3" s="4" t="n">
-        <v>46277.48446759259</v>
+        <v>46277.4872800926</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Mamba2_AC_Assault_seed6010_X</t>
+          <t>Mamba2_AC_Amidar_seed3710_X</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>ds19f3ml</t>
+          <t>s7qnin4f</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -1032,19 +1056,27 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Assault</t>
+          <t>Amidar</t>
         </is>
       </c>
       <c r="G4" s="3" t="n">
-        <v>6010</v>
+        <v>3710</v>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr"/>
-      <c r="J4" s="3" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>101.40</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>0.06</t>
+        </is>
+      </c>
       <c r="K4" s="3" t="n">
         <v>50000</v>
       </c>
@@ -1063,18 +1095,18 @@
         <v>0.0625</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>46277.48542824074</v>
+        <v>46277.51052083333</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Mamba2_AC_Amidar_seed6010_X</t>
+          <t>Mamba2_AC_Pong_seed2000_X</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>d2x1c1en</t>
+          <t>ldp9bu6i</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -1094,11 +1126,11 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Amidar</t>
+          <t>Pong</t>
         </is>
       </c>
       <c r="G5" s="3" t="n">
-        <v>6010</v>
+        <v>2000</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
@@ -1125,18 +1157,18 @@
         <v>0.0625</v>
       </c>
       <c r="P5" s="4" t="n">
-        <v>46277.4872800926</v>
+        <v>46277.51086805556</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Mamba2_AC_Amidar_seed3710_X</t>
+          <t>Mamba2_AC_BattleZone_seed3710_X</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>s7qnin4f</t>
+          <t>9l57kpp0</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -1156,7 +1188,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Amidar</t>
+          <t>BattleZone</t>
         </is>
       </c>
       <c r="G6" s="3" t="n">
@@ -1167,8 +1199,16 @@
           <t>X</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr"/>
-      <c r="J6" s="3" t="inlineStr"/>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>14000.00</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>0.33</t>
+        </is>
+      </c>
       <c r="K6" s="3" t="n">
         <v>50000</v>
       </c>
@@ -1187,18 +1227,18 @@
         <v>0.0625</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>46277.51052083333</v>
+        <v>46277.51194444444</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Mamba2_AC_Pong_seed2000_X</t>
+          <t>Mamba2_AC_Amidar_seed3710_O</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>ldp9bu6i</t>
+          <t>f2hapfd6</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -1218,19 +1258,27 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Pong</t>
+          <t>Amidar</t>
         </is>
       </c>
       <c r="G7" s="3" t="n">
-        <v>2000</v>
+        <v>3710</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr"/>
-      <c r="J7" s="3" t="inlineStr"/>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>105.20</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>0.06</t>
+        </is>
+      </c>
       <c r="K7" s="3" t="n">
         <v>50000</v>
       </c>
@@ -1249,18 +1297,18 @@
         <v>0.0625</v>
       </c>
       <c r="P7" s="4" t="n">
-        <v>46277.51086805556</v>
+        <v>46277.58818287037</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Mamba2_AC_BattleZone_seed3710_X</t>
+          <t>Mamba2_AC_BattleZone_seed3710_O</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>9l57kpp0</t>
+          <t>xjmo67zz</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -1288,11 +1336,19 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr"/>
-      <c r="J8" s="3" t="inlineStr"/>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>5800.00</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>0.10</t>
+        </is>
+      </c>
       <c r="K8" s="3" t="n">
         <v>50000</v>
       </c>
@@ -1311,18 +1367,18 @@
         <v>0.0625</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>46277.51194444444</v>
+        <v>46277.5909375</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Mamba2_AC_Amidar_seed3710_O</t>
+          <t>Mamba2_AC_Pong_seed2010_X</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>f2hapfd6</t>
+          <t>r7xx98gc</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -1342,18 +1398,22 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Amidar</t>
+          <t>Pong</t>
         </is>
       </c>
       <c r="G9" s="3" t="n">
-        <v>3710</v>
+        <v>2010</v>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="inlineStr"/>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>20.00</t>
+        </is>
+      </c>
       <c r="J9" s="3" t="inlineStr"/>
       <c r="K9" s="3" t="n">
         <v>50000</v>
@@ -1373,18 +1433,18 @@
         <v>0.0625</v>
       </c>
       <c r="P9" s="4" t="n">
-        <v>46277.58818287037</v>
+        <v>46277.63061342593</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Mamba2_AC_BattleZone_seed3710_O</t>
+          <t>Mamba2_AC_Assault_seed6010_O</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>xjmo67zz</t>
+          <t>cjat5h3s</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1404,18 +1464,22 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>BattleZone</t>
+          <t>Assault</t>
         </is>
       </c>
       <c r="G10" s="3" t="n">
-        <v>3710</v>
+        <v>6010</v>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr"/>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>630.00</t>
+        </is>
+      </c>
       <c r="J10" s="3" t="inlineStr"/>
       <c r="K10" s="3" t="n">
         <v>50000</v>
@@ -1435,18 +1499,18 @@
         <v>0.0625</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>46277.5909375</v>
+        <v>46277.66618055556</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Mamba2_AC_Pong_seed2010_X</t>
+          <t>Mamba2_AC_Amidar_seed6010_O</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>r7xx98gc</t>
+          <t>b7d1fcs6</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -1466,15 +1530,15 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Pong</t>
+          <t>Amidar</t>
         </is>
       </c>
       <c r="G11" s="3" t="n">
-        <v>2010</v>
+        <v>6010</v>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr"/>
@@ -1497,18 +1561,18 @@
         <v>0.0625</v>
       </c>
       <c r="P11" s="4" t="n">
-        <v>46277.63061342593</v>
+        <v>46277.66625</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Mamba2_AC_Krull_seed6010_O</t>
+          <t>Mamba2_AC_Pong_seed2000_O</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>jfobo71c</t>
+          <t>54peul18</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1528,11 +1592,11 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Krull</t>
+          <t>Pong</t>
         </is>
       </c>
       <c r="G12" s="3" t="n">
-        <v>6010</v>
+        <v>2000</v>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
@@ -1559,18 +1623,18 @@
         <v>0.0625</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>46277.66219907408</v>
+        <v>46277.70894675926</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Mamba2_AC_Frostbite_seed6010_O</t>
+          <t>Mamba2_AC_Qbert_seed3710_X</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>yek1u6ty</t>
+          <t>rdsp4vkd</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1590,19 +1654,27 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Frostbite</t>
+          <t>Qbert</t>
         </is>
       </c>
       <c r="G13" s="3" t="n">
-        <v>6010</v>
+        <v>3710</v>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr"/>
-      <c r="J13" s="3" t="inlineStr"/>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>787.50</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
       <c r="K13" s="3" t="n">
         <v>50000</v>
       </c>
@@ -1621,18 +1693,18 @@
         <v>0.0625</v>
       </c>
       <c r="P13" s="4" t="n">
-        <v>46277.66439814815</v>
+        <v>46277.78224537037</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Mamba2_AC_Assault_seed6010_O</t>
+          <t>Mamba2_AC_ChopperCommand_seed3710_X</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>cjat5h3s</t>
+          <t>wprgvkwu</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1652,19 +1724,27 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Assault</t>
+          <t>ChopperCommand</t>
         </is>
       </c>
       <c r="G14" s="3" t="n">
-        <v>6010</v>
+        <v>3710</v>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr"/>
-      <c r="J14" s="3" t="inlineStr"/>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>1250.00</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>0.07</t>
+        </is>
+      </c>
       <c r="K14" s="3" t="n">
         <v>50000</v>
       </c>
@@ -1683,18 +1763,18 @@
         <v>0.0625</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>46277.66618055556</v>
+        <v>46277.79376157407</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Mamba2_AC_Amidar_seed6010_O</t>
+          <t>Mamba2_AC_Pong_seed2010_O</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>b7d1fcs6</t>
+          <t>dbr7fc7u</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1714,18 +1794,22 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Amidar</t>
+          <t>Pong</t>
         </is>
       </c>
       <c r="G15" s="3" t="n">
-        <v>6010</v>
+        <v>2010</v>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr"/>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>20.00</t>
+        </is>
+      </c>
       <c r="J15" s="3" t="inlineStr"/>
       <c r="K15" s="3" t="n">
         <v>50000</v>
@@ -1745,18 +1829,18 @@
         <v>0.0625</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>46277.66625</v>
+        <v>46277.83049768519</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Mamba2_AC_Pong_seed2000_O</t>
+          <t>Mamba2_AC_Qbert_seed3710_O</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>54peul18</t>
+          <t>bwkx0q0r</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1776,19 +1860,27 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Pong</t>
+          <t>Qbert</t>
         </is>
       </c>
       <c r="G16" s="3" t="n">
-        <v>2000</v>
+        <v>3710</v>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr"/>
-      <c r="J16" s="3" t="inlineStr"/>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>792.50</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
       <c r="K16" s="3" t="n">
         <v>50000</v>
       </c>
@@ -1807,18 +1899,18 @@
         <v>0.0625</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>46277.70894675926</v>
+        <v>46277.86043981482</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Mamba2_AC_Qbert_seed3710_X</t>
+          <t>Mamba2_AC_ChopperCommand_seed3710_O</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>rdsp4vkd</t>
+          <t>nclj0x34</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1838,7 +1930,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Qbert</t>
+          <t>ChopperCommand</t>
         </is>
       </c>
       <c r="G17" s="3" t="n">
@@ -1846,17 +1938,17 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>787.50</t>
+          <t>1430.00</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>0.05</t>
+          <t>0.09</t>
         </is>
       </c>
       <c r="K17" s="3" t="n">
@@ -1877,18 +1969,18 @@
         <v>0.0625</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>46277.78224537037</v>
+        <v>46277.87179398148</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Mamba2_AC_ChopperCommand_seed3710_X</t>
+          <t>Mamba2_AC_Jamesbond_seed3710_X</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>wprgvkwu</t>
+          <t>6jiief14</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -1908,7 +2000,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>ChopperCommand</t>
+          <t>Jamesbond</t>
         </is>
       </c>
       <c r="G18" s="3" t="n">
@@ -1921,12 +2013,12 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>1250.00</t>
+          <t>355.00</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>0.07</t>
+          <t>1.19</t>
         </is>
       </c>
       <c r="K18" s="3" t="n">
@@ -1947,18 +2039,18 @@
         <v>0.0625</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>46277.79376157407</v>
+        <v>46278.05765046296</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Mamba2_AC_Pong_seed2010_O</t>
+          <t>Mamba2_AC_UpNDown_seed3710_X</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>dbr7fc7u</t>
+          <t>se3zzsqc</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1978,19 +2070,27 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Pong</t>
+          <t>UpNDown</t>
         </is>
       </c>
       <c r="G19" s="3" t="n">
-        <v>2010</v>
+        <v>3710</v>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="I19" s="3" t="inlineStr"/>
-      <c r="J19" s="3" t="inlineStr"/>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>2654.00</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>0.19</t>
+        </is>
+      </c>
       <c r="K19" s="3" t="n">
         <v>50000</v>
       </c>
@@ -2009,291 +2109,11 @@
         <v>0.0625</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>46277.83049768519</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Mamba2_AC_Qbert_seed3710_O</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>bwkx0q0r</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>finished</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>Mamba2</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>AC</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>Qbert</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="n">
-        <v>3710</v>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>792.50</t>
-        </is>
-      </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
-          <t>0.05</t>
-        </is>
-      </c>
-      <c r="K20" s="3" t="n">
-        <v>50000</v>
-      </c>
-      <c r="L20" s="3" t="inlineStr">
-        <is>
-          <t>retrieved</t>
-        </is>
-      </c>
-      <c r="M20" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="N20" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="O20" s="3" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="P20" s="4" t="n">
-        <v>46277.86043981482</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Mamba2_AC_ChopperCommand_seed3710_O</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>nclj0x34</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>finished</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Mamba2</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>AC</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>ChopperCommand</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="n">
-        <v>3710</v>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>1430.00</t>
-        </is>
-      </c>
-      <c r="J21" s="3" t="inlineStr">
-        <is>
-          <t>0.09</t>
-        </is>
-      </c>
-      <c r="K21" s="3" t="n">
-        <v>50000</v>
-      </c>
-      <c r="L21" s="3" t="inlineStr">
-        <is>
-          <t>retrieved</t>
-        </is>
-      </c>
-      <c r="M21" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="N21" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="O21" s="3" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="P21" s="4" t="n">
-        <v>46277.87179398148</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Mamba2_AC_Jamesbond_seed3710_X</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>6jiief14</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>finished</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>Mamba2</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>AC</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>Jamesbond</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="n">
-        <v>3710</v>
-      </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>355.00</t>
-        </is>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>1.19</t>
-        </is>
-      </c>
-      <c r="K22" s="3" t="n">
-        <v>50000</v>
-      </c>
-      <c r="L22" s="3" t="inlineStr">
-        <is>
-          <t>retrieved</t>
-        </is>
-      </c>
-      <c r="M22" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="N22" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="O22" s="3" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>46278.05765046296</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Mamba2_AC_UpNDown_seed3710_X</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>se3zzsqc</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>finished</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>Mamba2</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>AC</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>UpNDown</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="n">
-        <v>3710</v>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>2654.00</t>
-        </is>
-      </c>
-      <c r="J23" s="3" t="inlineStr">
-        <is>
-          <t>0.19</t>
-        </is>
-      </c>
-      <c r="K23" s="3" t="n">
-        <v>50000</v>
-      </c>
-      <c r="L23" s="3" t="inlineStr">
-        <is>
-          <t>retrieved</t>
-        </is>
-      </c>
-      <c r="M23" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="N23" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="O23" s="3" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="P23" s="4" t="n">
         <v>46278.08553240741</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P23"/>
+  <autoFilter ref="A1:P19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
a6000 job queue, 표 업뎃
</commit_message>
<xml_diff>
--- a/results/drama_results.xlsx
+++ b/results/drama_results.xlsx
@@ -840,12 +840,20 @@
           <t>X</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>220.00</t>
+        </is>
+      </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
       <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>870.00</t>
+        </is>
+      </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
           <t>281.00</t>
@@ -869,12 +877,20 @@
           <t>O</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>184.00</t>
+        </is>
+      </c>
       <c r="D11" s="3" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr"/>
       <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>339.00</t>
+        </is>
+      </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
           <t>268.00</t>
@@ -903,7 +919,11 @@
           <t>9400.00</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>16200.00</t>
+        </is>
+      </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr"/>
@@ -936,7 +956,11 @@
           <t>13600.00</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>9700.00</t>
+        </is>
+      </c>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr"/>
       <c r="G13" s="3" t="inlineStr"/>
@@ -1038,12 +1062,20 @@
           <t>X</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr"/>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>RUNNING</t>
+        </is>
+      </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>9.70</t>
+        </is>
+      </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
           <t>20.70</t>
@@ -1067,12 +1099,20 @@
           <t>O</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>17.70</t>
+        </is>
+      </c>
       <c r="D17" s="3" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr"/>
       <c r="G17" s="3" t="inlineStr"/>
-      <c r="H17" s="3" t="inlineStr"/>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>10.60</t>
+        </is>
+      </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
           <t>20.70</t>
@@ -1130,7 +1170,11 @@
           <t>1350.00</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr"/>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>RUNNING</t>
+        </is>
+      </c>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="inlineStr"/>
       <c r="G19" s="3" t="inlineStr"/>
@@ -1574,7 +1618,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr"/>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>580.00</t>
+        </is>
+      </c>
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr">
         <is>
@@ -1587,9 +1635,9 @@
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>RUNNING</t>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>1420.00</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr"/>
@@ -1607,7 +1655,11 @@
           <t>O</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr"/>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>600.00</t>
+        </is>
+      </c>
       <c r="D33" s="3" t="inlineStr"/>
       <c r="E33" s="3" t="inlineStr">
         <is>
@@ -1620,9 +1672,9 @@
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr"/>
-      <c r="H33" s="5" t="inlineStr">
-        <is>
-          <t>RUNNING</t>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>1140.00</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr"/>
@@ -1645,7 +1697,11 @@
           <t>8075.00</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>6783.00</t>
+        </is>
+      </c>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr"/>
       <c r="G34" s="2" t="inlineStr"/>
@@ -1678,9 +1734,9 @@
           <t>7926.00</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>RUNNING</t>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>8213.00</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr"/>
@@ -2198,7 +2254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P152"/>
+  <dimension ref="A1:P166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -12646,189 +12702,1177 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="7" t="inlineStr">
+      <c r="A150" s="3" t="inlineStr">
         <is>
           <t>Mamba2_AC_Krull_seed1710_O</t>
         </is>
       </c>
-      <c r="B150" s="7" t="inlineStr">
+      <c r="B150" s="3" t="inlineStr">
         <is>
           <t>hzj4baq1</t>
         </is>
       </c>
-      <c r="C150" s="7" t="inlineStr">
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>finished</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2</t>
+        </is>
+      </c>
+      <c r="E150" s="3" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="F150" s="3" t="inlineStr">
+        <is>
+          <t>Krull</t>
+        </is>
+      </c>
+      <c r="G150" s="3" t="n">
+        <v>1710</v>
+      </c>
+      <c r="H150" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="I150" s="3" t="inlineStr">
+        <is>
+          <t>8213.00</t>
+        </is>
+      </c>
+      <c r="J150" s="3" t="inlineStr">
+        <is>
+          <t>6.19</t>
+        </is>
+      </c>
+      <c r="K150" s="3" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L150" s="3" t="inlineStr">
+        <is>
+          <t>retrieved</t>
+        </is>
+      </c>
+      <c r="M150" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N150" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="O150" s="3" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="P150" s="6" t="n">
+        <v>46282.94171296297</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2_AC_Kangaroo_seed3710_O</t>
+        </is>
+      </c>
+      <c r="B151" s="3" t="inlineStr">
+        <is>
+          <t>7gg68i66</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>finished</t>
+        </is>
+      </c>
+      <c r="D151" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2</t>
+        </is>
+      </c>
+      <c r="E151" s="3" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="F151" s="3" t="inlineStr">
+        <is>
+          <t>Kangaroo</t>
+        </is>
+      </c>
+      <c r="G151" s="3" t="n">
+        <v>3710</v>
+      </c>
+      <c r="H151" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="I151" s="3" t="inlineStr">
+        <is>
+          <t>1140.00</t>
+        </is>
+      </c>
+      <c r="J151" s="3" t="inlineStr">
+        <is>
+          <t>0.36</t>
+        </is>
+      </c>
+      <c r="K151" s="3" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L151" s="3" t="inlineStr">
+        <is>
+          <t>retrieved</t>
+        </is>
+      </c>
+      <c r="M151" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N151" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="O151" s="3" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="P151" s="6" t="n">
+        <v>46283.06856481481</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2_AC_Krull_seed1710_X</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>c2qsumr8</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>finished</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2</t>
+        </is>
+      </c>
+      <c r="E152" s="3" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="F152" s="3" t="inlineStr">
+        <is>
+          <t>Krull</t>
+        </is>
+      </c>
+      <c r="G152" s="3" t="n">
+        <v>1710</v>
+      </c>
+      <c r="H152" s="3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I152" s="3" t="inlineStr">
+        <is>
+          <t>6783.00</t>
+        </is>
+      </c>
+      <c r="J152" s="3" t="inlineStr">
+        <is>
+          <t>4.85</t>
+        </is>
+      </c>
+      <c r="K152" s="3" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L152" s="3" t="inlineStr">
+        <is>
+          <t>retrieved</t>
+        </is>
+      </c>
+      <c r="M152" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N152" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="O152" s="3" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="P152" s="6" t="n">
+        <v>46283.0745949074</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2_AC_Kangaroo_seed3710_X</t>
+        </is>
+      </c>
+      <c r="B153" s="3" t="inlineStr">
+        <is>
+          <t>vvbxysmh</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>finished</t>
+        </is>
+      </c>
+      <c r="D153" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2</t>
+        </is>
+      </c>
+      <c r="E153" s="3" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="F153" s="3" t="inlineStr">
+        <is>
+          <t>Kangaroo</t>
+        </is>
+      </c>
+      <c r="G153" s="3" t="n">
+        <v>3710</v>
+      </c>
+      <c r="H153" s="3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I153" s="3" t="inlineStr">
+        <is>
+          <t>1420.00</t>
+        </is>
+      </c>
+      <c r="J153" s="3" t="inlineStr">
+        <is>
+          <t>0.46</t>
+        </is>
+      </c>
+      <c r="K153" s="3" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L153" s="3" t="inlineStr">
+        <is>
+          <t>retrieved</t>
+        </is>
+      </c>
+      <c r="M153" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N153" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="O153" s="3" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="P153" s="6" t="n">
+        <v>46283.19665509259</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2_AC_Kangaroo_seed710_O</t>
+        </is>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>mditu4ar</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>finished</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2</t>
+        </is>
+      </c>
+      <c r="E154" s="3" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="F154" s="3" t="inlineStr">
+        <is>
+          <t>Kangaroo</t>
+        </is>
+      </c>
+      <c r="G154" s="3" t="n">
+        <v>710</v>
+      </c>
+      <c r="H154" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="I154" s="3" t="inlineStr">
+        <is>
+          <t>600.00</t>
+        </is>
+      </c>
+      <c r="J154" s="3" t="inlineStr">
+        <is>
+          <t>0.18</t>
+        </is>
+      </c>
+      <c r="K154" s="3" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L154" s="3" t="inlineStr">
+        <is>
+          <t>retrieved</t>
+        </is>
+      </c>
+      <c r="M154" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N154" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="O154" s="3" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="P154" s="6" t="n">
+        <v>46283.22854166666</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2_AC_Kangaroo_seed710_X</t>
+        </is>
+      </c>
+      <c r="B155" s="3" t="inlineStr">
+        <is>
+          <t>xma3ku4y</t>
+        </is>
+      </c>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>finished</t>
+        </is>
+      </c>
+      <c r="D155" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2</t>
+        </is>
+      </c>
+      <c r="E155" s="3" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="F155" s="3" t="inlineStr">
+        <is>
+          <t>Kangaroo</t>
+        </is>
+      </c>
+      <c r="G155" s="3" t="n">
+        <v>710</v>
+      </c>
+      <c r="H155" s="3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I155" s="3" t="inlineStr">
+        <is>
+          <t>580.00</t>
+        </is>
+      </c>
+      <c r="J155" s="3" t="inlineStr">
+        <is>
+          <t>0.18</t>
+        </is>
+      </c>
+      <c r="K155" s="3" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L155" s="3" t="inlineStr">
+        <is>
+          <t>retrieved</t>
+        </is>
+      </c>
+      <c r="M155" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N155" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="O155" s="3" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="P155" s="6" t="n">
+        <v>46283.33405092593</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2_AC_BankHeist_seed3710_O</t>
+        </is>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>dlwj6ky3</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>finished</t>
+        </is>
+      </c>
+      <c r="D156" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2</t>
+        </is>
+      </c>
+      <c r="E156" s="3" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="F156" s="3" t="inlineStr">
+        <is>
+          <t>BankHeist</t>
+        </is>
+      </c>
+      <c r="G156" s="3" t="n">
+        <v>3710</v>
+      </c>
+      <c r="H156" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="I156" s="3" t="inlineStr">
+        <is>
+          <t>339.00</t>
+        </is>
+      </c>
+      <c r="J156" s="3" t="inlineStr">
+        <is>
+          <t>0.44</t>
+        </is>
+      </c>
+      <c r="K156" s="3" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L156" s="3" t="inlineStr">
+        <is>
+          <t>retrieved</t>
+        </is>
+      </c>
+      <c r="M156" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N156" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="O156" s="3" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="P156" s="6" t="n">
+        <v>46283.35032407408</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2_AC_BankHeist_seed710_O</t>
+        </is>
+      </c>
+      <c r="B157" s="3" t="inlineStr">
+        <is>
+          <t>ysny5opr</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>finished</t>
+        </is>
+      </c>
+      <c r="D157" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2</t>
+        </is>
+      </c>
+      <c r="E157" s="3" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="F157" s="3" t="inlineStr">
+        <is>
+          <t>BankHeist</t>
+        </is>
+      </c>
+      <c r="G157" s="3" t="n">
+        <v>710</v>
+      </c>
+      <c r="H157" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="I157" s="3" t="inlineStr">
+        <is>
+          <t>184.00</t>
+        </is>
+      </c>
+      <c r="J157" s="3" t="inlineStr">
+        <is>
+          <t>0.23</t>
+        </is>
+      </c>
+      <c r="K157" s="3" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L157" s="3" t="inlineStr">
+        <is>
+          <t>retrieved</t>
+        </is>
+      </c>
+      <c r="M157" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N157" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="O157" s="3" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="P157" s="6" t="n">
+        <v>46283.48784722222</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2_AC_BankHeist_seed3710_X</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>rr10cndm</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>finished</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2</t>
+        </is>
+      </c>
+      <c r="E158" s="3" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="F158" s="3" t="inlineStr">
+        <is>
+          <t>BankHeist</t>
+        </is>
+      </c>
+      <c r="G158" s="3" t="n">
+        <v>3710</v>
+      </c>
+      <c r="H158" s="3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I158" s="3" t="inlineStr">
+        <is>
+          <t>870.00</t>
+        </is>
+      </c>
+      <c r="J158" s="3" t="inlineStr">
+        <is>
+          <t>1.16</t>
+        </is>
+      </c>
+      <c r="K158" s="3" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L158" s="3" t="inlineStr">
+        <is>
+          <t>retrieved</t>
+        </is>
+      </c>
+      <c r="M158" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N158" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="O158" s="3" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="P158" s="6" t="n">
+        <v>46283.508125</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2_AC_BankHeist_seed710_X</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="inlineStr">
+        <is>
+          <t>p6nur6oq</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>finished</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2</t>
+        </is>
+      </c>
+      <c r="E159" s="3" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="F159" s="3" t="inlineStr">
+        <is>
+          <t>BankHeist</t>
+        </is>
+      </c>
+      <c r="G159" s="3" t="n">
+        <v>710</v>
+      </c>
+      <c r="H159" s="3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I159" s="3" t="inlineStr">
+        <is>
+          <t>220.00</t>
+        </is>
+      </c>
+      <c r="J159" s="3" t="inlineStr">
+        <is>
+          <t>0.28</t>
+        </is>
+      </c>
+      <c r="K159" s="3" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L159" s="3" t="inlineStr">
+        <is>
+          <t>retrieved</t>
+        </is>
+      </c>
+      <c r="M159" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N159" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="O159" s="3" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="P159" s="6" t="n">
+        <v>46283.64868055555</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2_AC_BattleZone_seed1710_O</t>
+        </is>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>jftlhvxb</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>finished</t>
+        </is>
+      </c>
+      <c r="D160" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2</t>
+        </is>
+      </c>
+      <c r="E160" s="3" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="F160" s="3" t="inlineStr">
+        <is>
+          <t>BattleZone</t>
+        </is>
+      </c>
+      <c r="G160" s="3" t="n">
+        <v>1710</v>
+      </c>
+      <c r="H160" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="I160" s="3" t="inlineStr">
+        <is>
+          <t>9700.00</t>
+        </is>
+      </c>
+      <c r="J160" s="3" t="inlineStr">
+        <is>
+          <t>0.21</t>
+        </is>
+      </c>
+      <c r="K160" s="3" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L160" s="3" t="inlineStr">
+        <is>
+          <t>retrieved</t>
+        </is>
+      </c>
+      <c r="M160" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N160" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="O160" s="3" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="P160" s="6" t="n">
+        <v>46283.6619212963</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2_AC_BattleZone_seed1710_X</t>
+        </is>
+      </c>
+      <c r="B161" s="3" t="inlineStr">
+        <is>
+          <t>iv87tu9s</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>finished</t>
+        </is>
+      </c>
+      <c r="D161" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2</t>
+        </is>
+      </c>
+      <c r="E161" s="3" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="F161" s="3" t="inlineStr">
+        <is>
+          <t>BattleZone</t>
+        </is>
+      </c>
+      <c r="G161" s="3" t="n">
+        <v>1710</v>
+      </c>
+      <c r="H161" s="3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I161" s="3" t="inlineStr">
+        <is>
+          <t>16200.00</t>
+        </is>
+      </c>
+      <c r="J161" s="3" t="inlineStr">
+        <is>
+          <t>0.40</t>
+        </is>
+      </c>
+      <c r="K161" s="3" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L161" s="3" t="inlineStr">
+        <is>
+          <t>retrieved</t>
+        </is>
+      </c>
+      <c r="M161" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N161" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="O161" s="3" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="P161" s="6" t="n">
+        <v>46283.76673611111</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2_AC_Breakout_seed3710_O</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>ynh2axz9</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>finished</t>
+        </is>
+      </c>
+      <c r="D162" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2</t>
+        </is>
+      </c>
+      <c r="E162" s="3" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="F162" s="3" t="inlineStr">
+        <is>
+          <t>Breakout</t>
+        </is>
+      </c>
+      <c r="G162" s="3" t="n">
+        <v>3710</v>
+      </c>
+      <c r="H162" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="I162" s="3" t="inlineStr">
+        <is>
+          <t>10.60</t>
+        </is>
+      </c>
+      <c r="J162" s="3" t="inlineStr">
+        <is>
+          <t>0.31</t>
+        </is>
+      </c>
+      <c r="K162" s="3" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L162" s="3" t="inlineStr">
+        <is>
+          <t>retrieved</t>
+        </is>
+      </c>
+      <c r="M162" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N162" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="O162" s="3" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="P162" s="6" t="n">
+        <v>46283.8025</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2_AC_Breakout_seed710_O</t>
+        </is>
+      </c>
+      <c r="B163" s="3" t="inlineStr">
+        <is>
+          <t>kpkgy63f</t>
+        </is>
+      </c>
+      <c r="C163" s="3" t="inlineStr">
+        <is>
+          <t>finished</t>
+        </is>
+      </c>
+      <c r="D163" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2</t>
+        </is>
+      </c>
+      <c r="E163" s="3" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="F163" s="3" t="inlineStr">
+        <is>
+          <t>Breakout</t>
+        </is>
+      </c>
+      <c r="G163" s="3" t="n">
+        <v>710</v>
+      </c>
+      <c r="H163" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="I163" s="3" t="inlineStr">
+        <is>
+          <t>17.70</t>
+        </is>
+      </c>
+      <c r="J163" s="3" t="inlineStr">
+        <is>
+          <t>0.56</t>
+        </is>
+      </c>
+      <c r="K163" s="3" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L163" s="3" t="inlineStr">
+        <is>
+          <t>retrieved</t>
+        </is>
+      </c>
+      <c r="M163" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N163" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="O163" s="3" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="P163" s="6" t="n">
+        <v>46283.92071759259</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2_AC_Breakout_seed3710_X</t>
+        </is>
+      </c>
+      <c r="B164" s="3" t="inlineStr">
+        <is>
+          <t>eb1idchp</t>
+        </is>
+      </c>
+      <c r="C164" s="3" t="inlineStr">
+        <is>
+          <t>finished</t>
+        </is>
+      </c>
+      <c r="D164" s="3" t="inlineStr">
+        <is>
+          <t>Mamba2</t>
+        </is>
+      </c>
+      <c r="E164" s="3" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="F164" s="3" t="inlineStr">
+        <is>
+          <t>Breakout</t>
+        </is>
+      </c>
+      <c r="G164" s="3" t="n">
+        <v>3710</v>
+      </c>
+      <c r="H164" s="3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I164" s="3" t="inlineStr">
+        <is>
+          <t>9.70</t>
+        </is>
+      </c>
+      <c r="J164" s="3" t="inlineStr">
+        <is>
+          <t>0.28</t>
+        </is>
+      </c>
+      <c r="K164" s="3" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L164" s="3" t="inlineStr">
+        <is>
+          <t>retrieved</t>
+        </is>
+      </c>
+      <c r="M164" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N164" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="O164" s="3" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="P164" s="6" t="n">
+        <v>46283.94190972222</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="7" t="inlineStr">
+        <is>
+          <t>Mamba2_AC_Breakout_seed710_X</t>
+        </is>
+      </c>
+      <c r="B165" s="7" t="inlineStr">
+        <is>
+          <t>foc79krr</t>
+        </is>
+      </c>
+      <c r="C165" s="7" t="inlineStr">
         <is>
           <t>running</t>
         </is>
       </c>
-      <c r="D150" s="7" t="inlineStr">
-        <is>
-          <t>Mamba2</t>
-        </is>
-      </c>
-      <c r="E150" s="7" t="inlineStr">
-        <is>
-          <t>AC</t>
-        </is>
-      </c>
-      <c r="F150" s="7" t="inlineStr">
-        <is>
-          <t>Krull</t>
-        </is>
-      </c>
-      <c r="G150" s="7" t="n">
+      <c r="D165" s="7" t="inlineStr">
+        <is>
+          <t>Mamba2</t>
+        </is>
+      </c>
+      <c r="E165" s="7" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="F165" s="7" t="inlineStr">
+        <is>
+          <t>Breakout</t>
+        </is>
+      </c>
+      <c r="G165" s="7" t="n">
+        <v>710</v>
+      </c>
+      <c r="H165" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I165" s="7" t="inlineStr"/>
+      <c r="J165" s="7" t="inlineStr"/>
+      <c r="K165" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L165" s="7" t="inlineStr">
+        <is>
+          <t>retrieved</t>
+        </is>
+      </c>
+      <c r="M165" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="N165" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="O165" s="7" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="P165" s="8" t="n">
+        <v>46284.05696759259</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="7" t="inlineStr">
+        <is>
+          <t>Mamba2_AC_ChopperCommand_seed1710_O</t>
+        </is>
+      </c>
+      <c r="B166" s="7" t="inlineStr">
+        <is>
+          <t>aimffgh0</t>
+        </is>
+      </c>
+      <c r="C166" s="7" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="D166" s="7" t="inlineStr">
+        <is>
+          <t>Mamba2</t>
+        </is>
+      </c>
+      <c r="E166" s="7" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="F166" s="7" t="inlineStr">
+        <is>
+          <t>ChopperCommand</t>
+        </is>
+      </c>
+      <c r="G166" s="7" t="n">
         <v>1710</v>
       </c>
-      <c r="H150" s="7" t="inlineStr">
+      <c r="H166" s="7" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="I150" s="7" t="inlineStr"/>
-      <c r="J150" s="7" t="inlineStr"/>
-      <c r="K150" s="7" t="n">
-        <v>50000</v>
-      </c>
-      <c r="L150" s="7" t="inlineStr">
-        <is>
-          <t>retrieved</t>
-        </is>
-      </c>
-      <c r="M150" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="N150" s="7" t="n">
-        <v>16</v>
-      </c>
-      <c r="O150" s="7" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="P150" s="8" t="n">
-        <v>46282.94171296297</v>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="7" t="inlineStr">
-        <is>
-          <t>Mamba2_AC_Kangaroo_seed3710_Both</t>
-        </is>
-      </c>
-      <c r="B151" s="7" t="inlineStr">
-        <is>
-          <t>h9dw46ew</t>
-        </is>
-      </c>
-      <c r="C151" s="7" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="D151" s="7" t="inlineStr">
-        <is>
-          <t>Mamba2</t>
-        </is>
-      </c>
-      <c r="E151" s="7" t="inlineStr">
-        <is>
-          <t>AC</t>
-        </is>
-      </c>
-      <c r="F151" s="7" t="inlineStr">
-        <is>
-          <t>Kangaroo</t>
-        </is>
-      </c>
-      <c r="G151" s="7" t="n">
-        <v>3710</v>
-      </c>
-      <c r="H151" s="7" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I151" s="7" t="inlineStr"/>
-      <c r="J151" s="7" t="inlineStr"/>
-      <c r="K151" s="7" t="n">
-        <v>50000</v>
-      </c>
-      <c r="L151" s="7" t="inlineStr">
-        <is>
-          <t>retrieved</t>
-        </is>
-      </c>
-      <c r="M151" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="N151" s="7" t="n">
-        <v>16</v>
-      </c>
-      <c r="O151" s="7" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="P151" s="8" t="n">
-        <v>46282.99206018518</v>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="7" t="inlineStr">
-        <is>
-          <t>Mamba2_AC_Kangaroo_seed3710_Both</t>
-        </is>
-      </c>
-      <c r="B152" s="7" t="inlineStr">
-        <is>
-          <t>h9dw46ew</t>
-        </is>
-      </c>
-      <c r="C152" s="7" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="D152" s="7" t="inlineStr">
-        <is>
-          <t>Mamba2</t>
-        </is>
-      </c>
-      <c r="E152" s="7" t="inlineStr">
-        <is>
-          <t>AC</t>
-        </is>
-      </c>
-      <c r="F152" s="7" t="inlineStr">
-        <is>
-          <t>Kangaroo</t>
-        </is>
-      </c>
-      <c r="G152" s="7" t="n">
-        <v>3710</v>
-      </c>
-      <c r="H152" s="7" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="I152" s="7" t="inlineStr"/>
-      <c r="J152" s="7" t="inlineStr"/>
-      <c r="K152" s="7" t="n">
-        <v>50000</v>
-      </c>
-      <c r="L152" s="7" t="inlineStr">
-        <is>
-          <t>retrieved</t>
-        </is>
-      </c>
-      <c r="M152" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="N152" s="7" t="n">
-        <v>16</v>
-      </c>
-      <c r="O152" s="7" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="P152" s="8" t="n">
-        <v>46282.99206018518</v>
+      <c r="I166" s="7" t="inlineStr"/>
+      <c r="J166" s="7" t="inlineStr"/>
+      <c r="K166" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L166" s="7" t="inlineStr">
+        <is>
+          <t>retrieved</t>
+        </is>
+      </c>
+      <c r="M166" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="N166" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="O166" s="7" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="P166" s="8" t="n">
+        <v>46284.09695601852</v>
       </c>
     </row>
   </sheetData>

</xml_diff>